<commit_message>
fix(led): 删 Intel NUC11 播控主机 — GK9000 双 HDMI 直接兼任
用户原始意图: GK9000 当时选 2×HDMI 就是为了直接驱动 LED 大屏,
NUC 是早期 seed 数据里的 over-design, 未经用户确认.

正确架构 (现确认):
- GK9000 HDMI 1 → NovaStar VX1000 (LED 视频源)
- GK9000 HDMI 2 → 监控/调试显示器
- 视频文件存 GK9000 D:\Media\, 跟智能控制系统在同一台机器
- GK9000 上跑 ViPlex Express 或 PotPlayer 做播放

改动:
- seed.service.ts: 删 LED-NUC-1 硬件条目, LED-CTRL-1 remark 更新
- EQUIPMENT_LIST 1.3: 删 LED-PLAYER-1 行, 增加方案说明
  · 采购总览 #8 (NUC) 改 "0", -¥4,000
  · 总价: ¥256,550 → ¥252,550
  · 主交换机端口分配 + 机柜布置同步更新
- GK9000_FIELD_SETUP §0: 显示项写明 "2×HDMI + DP/VGA"
- GK9000_FIELD_SETUP §6.5 新增: LED 视频播放配置
  · 接线 (HDMI1 接 VX1000, HDMI2 接监控屏)
  · Windows 显示设置 (扩展模式 + 分辨率)
  · 视频文件目录 D:\Media\ 结构
  · ViPlex Express vs PotPlayer/VLC 二选一方案
  · 开机自启脚本占位
- BOM Excel 3-LED大屏: 删 LED-PLAYER-1 行, 总计公式自动重算

净省 ¥4,000 + 1 IP + 1U 机柜空间 + 维护一台 Windows 工作量

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/printable/金湖展贸中心-设备BOM清单-2026-05-21.xlsx
+++ b/docs/printable/金湖展贸中心-设备BOM清单-2026-05-21.xlsx
@@ -4176,7 +4176,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4206,6 +4206,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -4323,7 +4324,7 @@
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>6.5M 像素 · 10×RJ45 · HDMI×2+DVI+SDI · 1U 机架</t>
+          <t>HDMI1 输入接 GK9000 中控主机 HDMI 输出 (省独立 NUC 播控主机). 6.5M 像素 · 10×RJ45 · HDMI×2+DVI+SDI · 1U 机架</t>
         </is>
       </c>
       <c r="K6" s="8" t="inlineStr">
@@ -4333,78 +4334,78 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>LED-PLAYER-1</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>3.2 LED 屏体配件 (按面积单独询价)</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="n"/>
+      <c r="C7" s="22" t="n"/>
+      <c r="D7" s="22" t="n"/>
+      <c r="E7" s="22" t="n"/>
+      <c r="F7" s="22" t="n"/>
+      <c r="G7" s="22" t="n"/>
+      <c r="H7" s="22" t="n"/>
+      <c r="I7" s="22" t="n"/>
+      <c r="J7" s="22" t="n"/>
+      <c r="K7" s="23" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>LED-RECV</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>LED</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>LED 播控主机 (媒体播放)</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>英特尔</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>Intel</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>NUC11</t>
-        </is>
-      </c>
-      <c r="G7" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" s="9" t="n">
-        <v>4000</v>
-      </c>
-      <c r="I7" s="9">
-        <f>G7*H7</f>
-        <v/>
-      </c>
-      <c r="J7" s="8" t="inlineStr">
-        <is>
-          <t>Win10 + ViPlex Express · HDMI 输出到 VX1000</t>
-        </is>
-      </c>
-      <c r="K7" s="8" t="inlineStr">
-        <is>
-          <t>1F 主控室机柜</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>3.2 LED 屏体配件 (按面积单独询价)</t>
-        </is>
-      </c>
-      <c r="B8" s="22" t="n"/>
-      <c r="C8" s="22" t="n"/>
-      <c r="D8" s="22" t="n"/>
-      <c r="E8" s="22" t="n"/>
-      <c r="F8" s="22" t="n"/>
-      <c r="G8" s="22" t="n"/>
-      <c r="H8" s="22" t="n"/>
-      <c r="I8" s="22" t="n"/>
-      <c r="J8" s="22" t="n"/>
-      <c r="K8" s="23" t="n"/>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>LED 接收卡 (按张计)</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>诺瓦星云</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>NovaStar</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>A4s / A8s</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="H8" s="9" t="n">
+        <v>200</v>
+      </c>
+      <c r="I8" s="9">
+        <f>G9*H9</f>
+        <v/>
+      </c>
+      <c r="J8" s="8" t="inlineStr">
+        <is>
+          <t>每张接 65 万像素 LED 模组, 数量按屏估算</t>
+        </is>
+      </c>
+      <c r="K8" s="8" t="inlineStr">
+        <is>
+          <t>屏幕内部</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>LED-RECV</t>
+          <t>LED-MODULE</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -4414,117 +4415,66 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>LED 接收卡 (按张计)</t>
+          <t>LED 显示模组 (按㎡计)</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>诺瓦星云</t>
+          <t>灯具厂家</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>NovaStar</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>A4s / A8s</t>
+          <t>按 P 间距选 P1.8/P2.5/P3</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="I9" s="9">
-        <f>G9*H9</f>
+        <f>G10*H10</f>
         <v/>
       </c>
       <c r="J9" s="8" t="inlineStr">
         <is>
-          <t>每张接 65 万像素 LED 模组, 数量按屏估算</t>
+          <t>AC 220V LED 模组, 按现场面积报价</t>
         </is>
       </c>
       <c r="K9" s="8" t="inlineStr">
         <is>
-          <t>屏幕内部</t>
+          <t>1F/2F 大屏区</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>LED-MODULE</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>LED</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>LED 显示模组 (按㎡计)</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>灯具厂家</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>按 P 间距选 P1.8/P2.5/P3</t>
-        </is>
-      </c>
-      <c r="G10" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H10" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="9">
-        <f>G10*H10</f>
-        <v/>
-      </c>
-      <c r="J10" s="8" t="inlineStr">
-        <is>
-          <t>AC 220V LED 模组, 按现场面积报价</t>
-        </is>
-      </c>
-      <c r="K10" s="8" t="inlineStr">
-        <is>
-          <t>1F/2F 大屏区</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>本表合计</t>
         </is>
       </c>
-      <c r="B11" s="22" t="n"/>
-      <c r="C11" s="22" t="n"/>
-      <c r="D11" s="22" t="n"/>
-      <c r="E11" s="22" t="n"/>
-      <c r="F11" s="22" t="n"/>
-      <c r="G11" s="22" t="n"/>
-      <c r="H11" s="23" t="n"/>
-      <c r="I11" s="20">
-        <f>SUM(I5:I10)</f>
-        <v/>
-      </c>
-      <c r="J11" s="21" t="n"/>
-      <c r="K11" s="21" t="n"/>
-    </row>
+      <c r="B10" s="22" t="n"/>
+      <c r="C10" s="22" t="n"/>
+      <c r="D10" s="22" t="n"/>
+      <c r="E10" s="22" t="n"/>
+      <c r="F10" s="22" t="n"/>
+      <c r="G10" s="22" t="n"/>
+      <c r="H10" s="23" t="n"/>
+      <c r="I10" s="20">
+        <f>SUM(I5:I9)</f>
+        <v/>
+      </c>
+      <c r="J10" s="21" t="n"/>
+      <c r="K10" s="21" t="n"/>
+    </row>
+    <row r="11" ht="24" customHeight="1"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A2:K2"/>
@@ -5062,7 +5012,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -5316,51 +5265,16 @@
           <t>HVAC-GW-2F</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>空调</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>2F TCP 集控网关</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>中弘</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>ZHONGHONG</t>
-        </is>
-      </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>B 集控网关 TCP 款</t>
-        </is>
-      </c>
-      <c r="G10" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H10" s="9" t="n">
-        <v>1200</v>
-      </c>
-      <c r="I10" s="9">
-        <f>G10*H10</f>
-        <v/>
-      </c>
-      <c r="J10" s="8" t="inlineStr">
-        <is>
-          <t>同上 · IP 192.168.50.52 · 挂 2F 外机 (12 内机 n=0..11)</t>
-        </is>
-      </c>
-      <c r="K10" s="8" t="inlineStr">
-        <is>
-          <t>2F 公共电箱 F201</t>
-        </is>
-      </c>
+      <c r="B10" s="22" t="n"/>
+      <c r="C10" s="22" t="n"/>
+      <c r="D10" s="22" t="n"/>
+      <c r="E10" s="22" t="n"/>
+      <c r="F10" s="22" t="n"/>
+      <c r="G10" s="22" t="n"/>
+      <c r="H10" s="22" t="n"/>
+      <c r="I10" s="22" t="n"/>
+      <c r="J10" s="22" t="n"/>
+      <c r="K10" s="23" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="18" t="inlineStr">
@@ -5853,51 +5767,16 @@
           <t>HVAC-1F-10</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>空调</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>空调内机 (企业综合展销区)</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>奥克斯</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>AUX</t>
-        </is>
-      </c>
-      <c r="F21" s="8" t="inlineStr">
-        <is>
-          <t>DLR-125F/DCDQH</t>
-        </is>
-      </c>
-      <c r="G21" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H21" s="9" t="n">
-        <v>5500</v>
-      </c>
-      <c r="I21" s="9">
-        <f>G20*H20</f>
-        <v/>
-      </c>
-      <c r="J21" s="8" t="inlineStr">
-        <is>
-          <t>2.2kW</t>
-        </is>
-      </c>
-      <c r="K21" s="8" t="inlineStr">
-        <is>
-          <t>1F 企业综合展销区</t>
-        </is>
-      </c>
+      <c r="B21" s="22" t="n"/>
+      <c r="C21" s="22" t="n"/>
+      <c r="D21" s="22" t="n"/>
+      <c r="E21" s="22" t="n"/>
+      <c r="F21" s="22" t="n"/>
+      <c r="G21" s="22" t="n"/>
+      <c r="H21" s="22" t="n"/>
+      <c r="I21" s="22" t="n"/>
+      <c r="J21" s="22" t="n"/>
+      <c r="K21" s="23" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="18" t="inlineStr">
@@ -6494,51 +6373,16 @@
           <t>HVAC-2F-22</t>
         </is>
       </c>
-      <c r="B34" s="7" t="inlineStr">
-        <is>
-          <t>空调</t>
-        </is>
-      </c>
-      <c r="C34" s="8" t="inlineStr">
-        <is>
-          <t>空调内机 (产业研究中心)</t>
-        </is>
-      </c>
-      <c r="D34" s="7" t="inlineStr">
-        <is>
-          <t>奥克斯</t>
-        </is>
-      </c>
-      <c r="E34" s="7" t="inlineStr">
-        <is>
-          <t>AUX</t>
-        </is>
-      </c>
-      <c r="F34" s="8" t="inlineStr">
-        <is>
-          <t>DLR-100F/DCDQH</t>
-        </is>
-      </c>
-      <c r="G34" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H34" s="9" t="n">
-        <v>4500</v>
-      </c>
-      <c r="I34" s="9">
-        <f>G33*H33</f>
-        <v/>
-      </c>
-      <c r="J34" s="8" t="inlineStr">
-        <is>
-          <t>2.2kW</t>
-        </is>
-      </c>
-      <c r="K34" s="8" t="inlineStr">
-        <is>
-          <t>2F 产业研究中心</t>
-        </is>
-      </c>
+      <c r="B34" s="22" t="n"/>
+      <c r="C34" s="22" t="n"/>
+      <c r="D34" s="22" t="n"/>
+      <c r="E34" s="22" t="n"/>
+      <c r="F34" s="22" t="n"/>
+      <c r="G34" s="22" t="n"/>
+      <c r="H34" s="22" t="n"/>
+      <c r="I34" s="22" t="n"/>
+      <c r="J34" s="22" t="n"/>
+      <c r="K34" s="23" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="18" t="inlineStr">
@@ -6563,37 +6407,13 @@
           <t>HVAC-CTRL</t>
         </is>
       </c>
-      <c r="B36" s="7" t="inlineStr">
-        <is>
-          <t>空调</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>触摸屏线控器</t>
-        </is>
-      </c>
-      <c r="D36" s="7" t="inlineStr">
-        <is>
-          <t>奥克斯</t>
-        </is>
-      </c>
-      <c r="E36" s="7" t="inlineStr">
-        <is>
-          <t>AUX</t>
-        </is>
-      </c>
-      <c r="F36" s="8" t="inlineStr">
-        <is>
-          <t>XK10-DL-AUX (内销)</t>
-        </is>
-      </c>
-      <c r="G36" s="7" t="n">
-        <v>22</v>
-      </c>
-      <c r="H36" s="9" t="n">
-        <v>200</v>
-      </c>
+      <c r="B36" s="22" t="n"/>
+      <c r="C36" s="22" t="n"/>
+      <c r="D36" s="22" t="n"/>
+      <c r="E36" s="22" t="n"/>
+      <c r="F36" s="22" t="n"/>
+      <c r="G36" s="22" t="n"/>
+      <c r="H36" s="23" t="n"/>
       <c r="I36" s="9">
         <f>G35*H35</f>
         <v/>

</xml_diff>